<commit_message>
Add schedule, presenter hover, last-updated badge; auto-convert intro.docx
- Read FANT26_schedule.xlsx (Schedule + Presentors sheets) in build.py;
  pass schedule data to both HTML and PDF templates
- Website: schedule table with presenter chips that show topic on hover;
  last-updated badge in the header meta line
- PDF: schedule page (after TOC) with presenters and topics listed per slot
- build.py: for DE intro, mammoth-converts intro.html.docx on the fly so
  the CI always renders the latest docx without manual HTML updates
- Add openpyxl and mammoth to requirements.txt
- Add schedule_heading / presenters_label / last_updated keys to i18n

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/FANT26_merged.xlsx
+++ b/data/FANT26_merged.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="1" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3234" yWindow="3234" windowWidth="17280" windowHeight="9984" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="FANT26 merged" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -50,7 +49,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -414,7 +413,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:X12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83984375" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
Update data files: merged submissions, schedule, intro text
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/FANT26_merged.xlsx
+++ b/data/FANT26_merged.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="1" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3234" yWindow="3234" windowWidth="17280" windowHeight="9984" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3264" yWindow="3264" windowWidth="17280" windowHeight="9984" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="FANT26 merged" sheetId="1" state="visible" r:id="rId1"/>
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X12"/>
+  <dimension ref="A1:X14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83984375" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -780,12 +780,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Obeng Mensah &amp; Fäder</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Deborah &amp; Eymard</t>
+          <t>Obeng Mensah, Deborah &amp; Fäder, Eymard</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1171,6 +1166,85 @@
       <c r="S12" t="inlineStr">
         <is>
           <t>Archaeological research in Egypt’s desert regions has faced significant challenges in recent years due to regional and global constraints. Despite these difficulties, close collaboration with local partners has enabled joint initiatives in both research and academic training. This contribution provides an overview of archaeological projects and activities conducted by the University of Cologne in the Western Desert of Egypt over the past years and discusses future perspectives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Gestrich</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Nick</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Goethe Universität Frankfurt</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>New archaeological fieldwork in the Tagant, Mauritania: The end of the Tichitt tradition?</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>The Late Stone Age Tichitt complex is famous (among archaeologists of West Africa, at least) for its early and large stone-built settlements, indications of social complexity, and settled agro-pastoral lifeways. At the same time, research has been rather sparsely spread over its large, densely settled area. Many of the key questions remain essentially unanswered. The Tagant, to the west of the Tichitt complex' core area, is often cited as having continued the Tichitt tradition beyond its end in the mid-first millennium BCE. However, the entire region has only been subject of fieldwork for a single PhD thesis in the early 1990s. Since then, satellite surveys have been carried out, which provide only limited information. This paper reports on first results of a restudy of materials and a short survey campaign, as well as giving a preview of future planned work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Puerta Schardt</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Juan-Marco</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Doctoral candidate</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Goethe Universität Frankfurt</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Provenance analysis of clay smoking pipes in West Africa using pXRF</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update FANT26_merged.xlsx with latest submissions
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/FANT26_merged.xlsx
+++ b/data/FANT26_merged.xlsx
@@ -1170,6 +1170,11 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026/05/16 1:24:35 AM OESZ</t>
+        </is>
+      </c>
       <c r="B13" t="inlineStr">
         <is>
           <t>Gestrich</t>
@@ -1212,6 +1217,11 @@
       </c>
     </row>
     <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026/05/16 1:24:35 AM OESZ</t>
+        </is>
+      </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>Puerta Schardt</t>

</xml_diff>

<commit_message>
Update FANT26_merged.xlsx: add Puerta Schardt contribution
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/FANT26_merged.xlsx
+++ b/data/FANT26_merged.xlsx
@@ -45,8 +45,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1210,6 +1213,11 @@
           <t>New archaeological fieldwork in the Tagant, Mauritania: The end of the Tichitt tradition?</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Mauretania, Tichitt, Tagant, Settlements, Agropastoralism</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr">
         <is>
           <t>The Late Stone Age Tichitt complex is famous (among archaeologists of West Africa, at least) for its early and large stone-built settlements, indications of social complexity, and settled agro-pastoral lifeways. At the same time, research has been rather sparsely spread over its large, densely settled area. Many of the key questions remain essentially unanswered. The Tagant, to the west of the Tichitt complex' core area, is often cited as having continued the Tichitt tradition beyond its end in the mid-first millennium BCE. However, the entire region has only been subject of fieldwork for a single PhD thesis in the early 1990s. Since then, satellite surveys have been carried out, which provide only limited information. This paper reports on first results of a restudy of materials and a short survey campaign, as well as giving a preview of future planned work.</t>
@@ -1257,8 +1265,14 @@
           <t>Provenance analysis of clay smoking pipes in West Africa using pXRF</t>
         </is>
       </c>
+      <c r="S14" s="1" t="inlineStr">
+        <is>
+          <t>From around 1600 CE, clay smoking pipes become a regular component of West African site assemblages, yet they routinely differ from the accompanying pottery in both fabric and decoration. We apply pXRF to pipes and local pottery from 5 different sites, using the potteries geochemical signature as a baseline against which pipe provenance can be assessed to get a better inside on the relation between pipe and pottery production.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add roundtable entry to FANT26_merged.xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/FANT26_merged.xlsx
+++ b/data/FANT26_merged.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X14"/>
+  <dimension ref="A1:X15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83984375" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -817,16 +817,6 @@
           <t>Deborah Obeng Mensah, Eymard Fäder</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Deborah Obeng Mensah</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Eymard Fäder</t>
-        </is>
-      </c>
       <c r="R6" t="inlineStr">
         <is>
           <t>3D imaging, digital archives, cultural heritage preservation</t>
@@ -1265,9 +1255,46 @@
           <t>Provenance analysis of clay smoking pipes in West Africa using pXRF</t>
         </is>
       </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Umar Musa</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Patrick Quinn</t>
+        </is>
+      </c>
       <c r="S14" s="1" t="inlineStr">
         <is>
           <t>From around 1600 CE, clay smoking pipes become a regular component of West African site assemblages, yet they routinely differ from the accompanying pottery in both fabric and decoration. We apply pXRF to pipes and local pottery from 5 different sites, using the potteries geochemical signature as a baseline against which pipe provenance can be assessed to get a better inside on the relation between pipe and pottery production.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Goethe Universität Frankfurt</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Roundtable</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Archaeometrical methods in African archaoelogy</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>Archaeometric methods play an increasingly important role in African archaeology, allowing us to extract from archaeological materials a wealth of information on knowledge and skills, trade, and use that is not accessible to the naked eye. These methods differ considerably in terms of effort and the insights they yield. What they share, however, is the need for the research question, sampling strategy, data management, and data analysis to be carefully considered and aligned with one another.This roundtable offers an overview of different archaeometric approaches and a discussion of their opportunities and challenges. Which archaeometric questions and methods are currently relevant? What resources and capacities do we have, and how can we expand or connect them? How can archaeometric projects be designed together with African partners?</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update FANT26_merged.xlsx and FANT26_schedule.xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/FANT26_merged.xlsx
+++ b/data/FANT26_merged.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3264" yWindow="3264" windowWidth="17280" windowHeight="9984" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3600" yWindow="3600" windowWidth="17280" windowHeight="9984" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="FANT26 merged" sheetId="1" state="visible" r:id="rId1"/>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X15"/>
+  <dimension ref="A1:X17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83984375" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -1272,6 +1272,11 @@
       </c>
     </row>
     <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026/05/16 1:24:35 AM OESZ</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>Goethe Universität Frankfurt</t>
@@ -1295,6 +1300,105 @@
       <c r="X15" t="inlineStr">
         <is>
           <t>Archaeometric methods play an increasingly important role in African archaeology, allowing us to extract from archaeological materials a wealth of information on knowledge and skills, trade, and use that is not accessible to the naked eye. These methods differ considerably in terms of effort and the insights they yield. What they share, however, is the need for the research question, sampling strategy, data management, and data analysis to be carefully considered and aligned with one another.This roundtable offers an overview of different archaeometric approaches and a discussion of their opportunities and challenges. Which archaeometric questions and methods are currently relevant? What resources and capacities do we have, and how can we expand or connect them? How can archaeometric projects be designed together with African partners?</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026/05/16 1:24:35 AM OESZ</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Höhn</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Alexa</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Goethe Universität Frankfurt</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Präsentation</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Die archäobotanischen Vergleichssammlungen an der Goethe-Universität, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Sammlungen, Westafrika, Archäobotanik</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Vergleichssammlungen sind eine unverzichtbare Grundlage in archäobotanischer Forschung und Lehre. An der Goethe-Universität umfassen sie Hölzer, Pollen, Früchte, Samen und Phytolithen. Insbesondere die umfangreichen westafrikanischen Bestände stellen eine international bedeutende Ressource dar und werden regelmäßig von Gastwissenschaftlerinnen und Gastwissenschaftlern genutzt. Im Rahmen der Objektdatenbank CODA werden die Sammlungen systematisch digital erschlossen, um ihre wissenschaftliche Nutzung weltweit zu erleichtern. Zugleich dokumentieren die Objekte Umwelt, Kultur- und Kolonialgeschichte und besitzen damit einen eigenständigen Quellenwert für interdisziplinäre Forschung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Magnavita</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Sonja</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Goethe Universität Frankfurt</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Trans-Sudanic vs. Trans-Saharan contacts: chemical analysis of glass beads from Kanem, Chad</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>glass, beads, Kanem, archaeometry</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>This talk presents the results of archaeometric analyses of a collection of 12th-14th century glass beads from the archaeological site of Tié (Chad) — the presumed capital of the early Kanem Empire northeast of Lake Chad. The appearance, manufacture, and chemical composition of the beads largely correspond to those of glass beads that were in circulation in the Indian Ocean region, suggesting a connection between Kanem and East or Northeast Africa. In light of the finds from Kanem, a trade route along the savanna belt seems more plausible than a trans-Saharan route, especially when other glass bead finds from the continent are taken into account as well.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update FANT26_merged.xlsx (email address correction)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/FANT26_merged.xlsx
+++ b/data/FANT26_merged.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\FANT_2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BCAE054-BABF-4364-B490-C031A14274F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2833A93A-D178-4557-8F55-B7F518492C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="152">
   <si>
     <t>Zeitstempel</t>
   </si>
@@ -477,6 +477,9 @@
   </si>
   <si>
     <t>Maximilian</t>
+  </si>
+  <si>
+    <t>Maximilian_schulze97@t-online.de</t>
   </si>
 </sst>
 </file>
@@ -1524,6 +1527,9 @@
       <c r="E19" t="s">
         <v>76</v>
       </c>
+      <c r="F19" t="s">
+        <v>151</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>